<commit_message>
Update agent asset metadata and camera motor inventory data
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/attached_assets/cam-motors/cam-motors-inventory-import.xlsx
+++ b/attached_assets/cam-motors/cam-motors-inventory-import.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="139">
   <si>
     <t>Inventory ID</t>
   </si>
@@ -91,12 +91,18 @@
     <t/>
   </si>
   <si>
+    <t>LVCRNVTGYKUMCG1TS</t>
+  </si>
+  <si>
     <t>Foton</t>
   </si>
   <si>
     <t>Tunland G7</t>
   </si>
   <si>
+    <t>ENB07XYHVSSGNCE9U</t>
+  </si>
+  <si>
     <t>Diesel</t>
   </si>
   <si>
@@ -118,10 +124,16 @@
     <t>yes</t>
   </si>
   <si>
+    <t>L1CLVK5DKV60VT3DC</t>
+  </si>
+  <si>
     <t>Jetour</t>
   </si>
   <si>
     <t>DASHING</t>
+  </si>
+  <si>
+    <t>ENWXL220MK2VRU592</t>
   </si>
   <si>
     <t>Petrol</t>
@@ -143,7 +155,13 @@
     <t>no</t>
   </si>
   <si>
+    <t>L1CKBSE7NEV3XFY6J</t>
+  </si>
+  <si>
     <t>T2</t>
+  </si>
+  <si>
+    <t>EN8YCCSWWBEN1HHA1</t>
   </si>
   <si>
     <t>https://cammotors.gy/api/storage/objects/c4feaef0-e79f-43fe-b9df-26232c6fb9d4</t>
@@ -156,7 +174,13 @@
 Rugged / Hardcore Adventure SUV Available colors: Black, White, Silver, Electroplated Green, Highway Grey.</t>
   </si>
   <si>
+    <t>L1CF3XL3H0BR0DN31</t>
+  </si>
+  <si>
     <t>T1</t>
+  </si>
+  <si>
+    <t>EN79RJFRAMBMKBR1U</t>
   </si>
   <si>
     <t>https://cammotors.gy/api/storage/objects/365ace40-3126-4595-85d5-7fd86bbe8efb</t>
@@ -169,9 +193,15 @@
 Time to Awaken — Lite Off-Road SUV Available colors: Black, white, Silver, Electroplated Green.</t>
   </si>
   <si>
+    <t>LVCBYVHA77VGYFU3T</t>
+  </si>
+  <si>
     <t>Tunland V9</t>
   </si>
   <si>
+    <t>ENSU1V1A40C3Y1W9R</t>
+  </si>
+  <si>
     <t>https://cammotors.gy/api/storage/objects/d33b040a-45db-432a-a822-2cf195a3f992</t>
   </si>
   <si>
@@ -181,9 +211,15 @@
     <t>A robust, full-size hybrid pickup truck, the Foton Tunland V9 has a 2.0-litre turbocharged diesel engine with a 48V mild-hybrid system that generates about 161 horsepower and 450 Nm of torque. It is mated to an 8-speed automatic transmission. It has a roomy cabin with contemporary technology, such as a 12.3-inch digital display and a 14.6-inch infotainment screen, and a smooth ride akin to an SUV thanks to its coil-sprung multi-link rear suspension. Key features: Rugged exterior design; Off-road suspension; Luxurious interior; Smart connectivity and modern technology; Full-size body.</t>
   </si>
   <si>
+    <t>LVCW0YWZS151SXRM1</t>
+  </si>
+  <si>
     <t>Aumark S Flatbed or Tray</t>
   </si>
   <si>
+    <t>EN18J5YBNAWU1HBSZ</t>
+  </si>
+  <si>
     <t>Light Duty Truck</t>
   </si>
   <si>
@@ -199,9 +235,15 @@
     <t>A family of light-duty commercial vehicles built for versatility in urban and distribution operations, with reliable Cummins or Perkins powertrains, ZF or other gearboxes, and a strong safety focus including full air braking and crash-compliant cabins. Available in tipper, dry box, and refrigerated configurations with driver-centric, ergonomic cabins. Key features: Comfort Cabin; Air-Assisted Brakes and Clutch; Cab design for Great Visibility; Compact body suitable for urban Areas.</t>
   </si>
   <si>
+    <t>L1C9CPXUHDN3X4E1U</t>
+  </si>
+  <si>
     <t>X70 PLUS(X70P)</t>
   </si>
   <si>
+    <t>ENH76E3EEC4N0FEH4</t>
+  </si>
+  <si>
     <t>White</t>
   </si>
   <si>
@@ -211,9 +253,15 @@
     <t>https://cammotors.gy/api/storage/objects/56e5faad-2219-44c7-8d79-1d5eab79c02f, https://cammotors.gy/api/storage/objects/71610bdd-5fce-4e8d-a8e2-17fd44492483, https://cammotors.gy/api/storage/objects/4da8d525-71e6-4ce3-a073-ff331f1edd44, https://cammotors.gy/api/storage/objects/02c20099-cfbc-4f3e-8b98-c82e5deda968, https://cammotors.gy/api/storage/objects/c63e85d9-5476-4094-bdfc-d70c1fdb9709, https://cammotors.gy/api/storage/objects/34195dbb-93d1-4527-b149-2643d79ed0fb, https://cammotors.gy/api/storage/objects/1274bdd2-e9c4-4529-863d-bdf3212a15cd, https://cammotors.gy/api/storage/objects/f9391772-3663-43d2-99f7-9ccf44a510b5, https://cammotors.gy/api/storage/objects/9b7775c6-7298-4932-ba71-e439fd5c6a16, https://cammotors.gy/api/storage/objects/a76b69d3-847c-4136-a71e-34e6a78af1c8, https://cammotors.gy/api/storage/objects/fff65ff3-c0e8-4370-b2f7-0eb9c67bcbf1, https://cammotors.gy/api/storage/objects/709aaa84-a6f5-4710-8221-d311ca984c71, https://cammotors.gy/api/storage/objects/bec97c74-1dbd-4aba-8b76-be059e9e9a7c</t>
   </si>
   <si>
+    <t>LVCEC2F96VEEWED2X</t>
+  </si>
+  <si>
     <t>Aumark S Dry Van Box</t>
   </si>
   <si>
+    <t>ENFNV1MJSPNL0VPS0</t>
+  </si>
+  <si>
     <t>https://cammotors.gy/api/storage/objects/fd67eec8-8b5e-4d67-9719-b6cc1b1438e9</t>
   </si>
   <si>
@@ -223,18 +271,30 @@
     <t>The Foton Aumark S is a family of light-duty commercial vehicles built for versatility in urban and distribution operations, with reliable powertrains from Cummins or Perkins, ZF or other gears, and a strong focus on safety with features like full air braking and crash-compliant cabins. Aumark S trucks, which are well-known for their driver-centric, ergonomic cabins with contemporary technology and fast handling, provide a range of configurations to suit different company requirements, such as tipper, dry box, and refrigerated applications. Key features: Comfort Cabin; Air-Assisted Brakes and Clutch; Cab design for Great Visibility; Compact body suitable for urban Areas.</t>
   </si>
   <si>
+    <t>LVCP3KEFEN1M5Z53R</t>
+  </si>
+  <si>
     <t>Aumark S Refrigerator Box</t>
   </si>
   <si>
+    <t>EN6RWNHHUECHA6NWN</t>
+  </si>
+  <si>
     <t>https://cammotors.gy/api/storage/objects/0127ec2c-7426-4a84-b0a1-e32891cdf3c7</t>
   </si>
   <si>
     <t>https://cammotors.gy/api/storage/objects/0127ec2c-7426-4a84-b0a1-e32891cdf3c7, https://cammotors.gy/api/storage/objects/40c2c2ef-0499-4db4-a6d7-df6968dfc91c, https://cammotors.gy/api/storage/objects/896ab1af-20f9-403a-b247-191308fd5fab, https://cammotors.gy/api/storage/objects/f9d731f5-aa8c-4f05-8f4d-8e7ad04c8922, https://cammotors.gy/api/storage/objects/8799a680-1ab9-4726-a66e-959567b4fbba, https://cammotors.gy/api/storage/objects/570bf653-f16b-4d1b-85a2-3e59430d3dd8, https://cammotors.gy/api/storage/objects/cf52e872-6a69-4639-a173-2b22c5614f46, https://cammotors.gy/api/storage/objects/b5a9666c-f668-403a-bd7f-6cf1c128d916, https://cammotors.gy/api/storage/objects/002e8255-900f-4bfd-9384-cfd6cceaf7bf</t>
   </si>
   <si>
+    <t>LVCRTZGY0GDBJ6UF1</t>
+  </si>
+  <si>
     <t>Miler Flatbed or Tray</t>
   </si>
   <si>
+    <t>EN4PCB3X5K9YGJ621</t>
+  </si>
+  <si>
     <t>https://cammotors.gy/api/storage/objects/13df5669-c4b5-4047-843e-22cdbc260e3d</t>
   </si>
   <si>
@@ -244,9 +304,15 @@
     <t>For companies that appreciate dependability and adaptability, the Foton Miler Range Truck is the best option. Its open flatbed design provides unparalleled adaptability, easily handling big, enormous, and irregular cargo, and is designed to accommodate a range of transportation needs. Key features: Lightweight Compact Body; Fuel Efficient; Fits in narrow roadways; Easy to maneuver in congested traffic areas.</t>
   </si>
   <si>
+    <t>LVCSGEJ9USL1RZLTE</t>
+  </si>
+  <si>
     <t>Miler Dry Van Box</t>
   </si>
   <si>
+    <t>ENMDZJFW4XH16BM9N</t>
+  </si>
+  <si>
     <t>Miler</t>
   </si>
   <si>
@@ -256,18 +322,30 @@
     <t>https://cammotors.gy/api/storage/objects/5b2e73dd-a56b-4f5f-b5a9-cd57dd8a2b14, https://cammotors.gy/api/storage/objects/103c790b-aae5-4fdf-b1d8-0ebdcfd61973, https://cammotors.gy/api/storage/objects/13893971-39f1-4a6b-92a3-facc3097217a, https://cammotors.gy/api/storage/objects/60efb2f9-8573-439d-9d24-35600498f646, https://cammotors.gy/api/storage/objects/14c35e46-cdf3-4e10-aecb-a2448ada764d</t>
   </si>
   <si>
+    <t>LVCA9VC7Y7FLB0H1P</t>
+  </si>
+  <si>
     <t>Miler Refrigerator Box</t>
   </si>
   <si>
+    <t>ENJ7HX5M389GPYTBJ</t>
+  </si>
+  <si>
     <t>https://cammotors.gy/api/storage/objects/9f6f072f-bbc9-4fff-bcaa-97fe53214cf2</t>
   </si>
   <si>
     <t>https://cammotors.gy/api/storage/objects/9f6f072f-bbc9-4fff-bcaa-97fe53214cf2, https://cammotors.gy/api/storage/objects/b8723264-97d2-4e44-8f5f-85c5d08c7077, https://cammotors.gy/api/storage/objects/3ba3169e-d89c-440f-92e3-303c99cc40e4, https://cammotors.gy/api/storage/objects/3d87cbde-c5ed-4172-a5fb-fc1e3c45b864</t>
   </si>
   <si>
+    <t>LVC22AFZJP1S5G2PS</t>
+  </si>
+  <si>
     <t>View C2 Panel Van</t>
   </si>
   <si>
+    <t>ENJFTH7TR3XP4FJB8</t>
+  </si>
+  <si>
     <t>Van</t>
   </si>
   <si>
@@ -283,9 +361,15 @@
     <t>The most recent turbocharger intake system is seen in the View CS2. The highest performance is guaranteed by BOSCH's electronically regulated, high-pressure common rail fuel injection system. A modular design idea serves as the foundation for the powertrain. Compared to other comparable products, it contains 40% fewer components. Key features: Suitable for multi-use, Passenger, Cargo and can be used as a Utility Van, or a cargo van.; Sturdy Suspension, Robust and efficient Diesel Engine..</t>
   </si>
   <si>
+    <t>LVC1AWGKUNSY24YDM</t>
+  </si>
+  <si>
     <t>View CS2 Passenger Bus</t>
   </si>
   <si>
+    <t>EN0S3EDMAJBJKN2VD</t>
+  </si>
+  <si>
     <t>View CS2</t>
   </si>
   <si>
@@ -295,9 +379,15 @@
     <t>https://cammotors.gy/api/storage/objects/91226520-1a38-4132-8301-73bfd52815f9, https://cammotors.gy/api/storage/objects/03f1bcff-61ab-4b7f-8a18-f3131d847252, https://cammotors.gy/api/storage/objects/bdfd2b53-601c-480f-8018-b336d1ddd845, https://cammotors.gy/api/storage/objects/596efc4a-dacd-4929-90fa-8187346fb28b, https://cammotors.gy/api/storage/objects/d3ac6c3b-6605-4e7f-a874-e29dcdf85165, https://cammotors.gy/api/storage/objects/4f0672ca-d959-4795-ab4c-ac375107c694, https://cammotors.gy/api/storage/objects/77ea17fd-acbe-400a-a116-35feedd4bfdd</t>
   </si>
   <si>
+    <t>LVCHVRFRNPC2G64TZ</t>
+  </si>
+  <si>
     <t>Truck Mate Flatbed/Tray</t>
   </si>
   <si>
+    <t>ENWN85V4XTHU3KUS6</t>
+  </si>
+  <si>
     <t>Mini Truck</t>
   </si>
   <si>
@@ -313,16 +403,28 @@
     <t>A light-duty truck that is inexpensive, dependable, and adaptable, the Foton Truck Mate is made to help businesses, especially small and medium-sized. It is appropriate for a range of uses, including deliveries, trades, and mobile services. Key features: Agility, Multi-Purpose Use; Convenient for downtown distribution and delivery; Great for Mobile Business, fuel-efficient; Very economical to operate.</t>
   </si>
   <si>
+    <t>LVCPCUNCSHJWKUMV5</t>
+  </si>
+  <si>
     <t>Truck Mate Dry Van Box</t>
   </si>
   <si>
+    <t>END2TJBGL4PBYH098</t>
+  </si>
+  <si>
     <t>https://cammotors.gy/api/storage/objects/acfb24aa-77cf-4be5-befb-149cb52eb971</t>
   </si>
   <si>
     <t>https://cammotors.gy/api/storage/objects/acfb24aa-77cf-4be5-befb-149cb52eb971, https://cammotors.gy/api/storage/objects/f2f2c270-2144-4101-b5d7-7a75f0d03436, https://cammotors.gy/api/storage/objects/3dd4c8a9-6f6a-48f7-b6e5-5322ea359425, https://cammotors.gy/api/storage/objects/d3a6b55e-a90d-4bdc-b40c-79f8ce71e128, https://cammotors.gy/api/storage/objects/836350c0-79da-4ca6-b423-ba56ab0927bf, https://cammotors.gy/api/storage/objects/a4f25335-008b-4c50-9ea9-29bbbea6c8c5, https://cammotors.gy/api/storage/objects/c8104d0f-e326-4f1a-8ece-288920592056, https://cammotors.gy/api/storage/objects/b7856ce6-0b92-44c5-be59-af98e5b765e1, https://cammotors.gy/api/storage/objects/0e0495ba-663f-4c7c-80fa-0eb9e3f88a97, https://cammotors.gy/api/storage/objects/46384f4a-0cf2-4cf9-a51a-ed9a4005e9b3, https://cammotors.gy/api/storage/objects/1bbb1922-ff54-447a-b948-f930c2c29834, https://cammotors.gy/api/storage/objects/828c54e7-73fd-47e8-8009-5d9465179f7a, https://cammotors.gy/api/storage/objects/aa5c1948-8fac-4242-83d4-f08043322369, https://cammotors.gy/api/storage/objects/502cde39-5316-430b-af58-9a0c455cb4f5</t>
   </si>
   <si>
+    <t>LVCBTX1AD8D3V5ZAC</t>
+  </si>
+  <si>
     <t>Truck Mate Refrigerator Box</t>
+  </si>
+  <si>
+    <t>ENBT0CZEESR69DYA3</t>
   </si>
   <si>
     <t>https://cammotors.gy/api/storage/objects/20f063af-0030-4d7c-b81f-d345f67a918c</t>
@@ -797,13 +899,13 @@
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
         <v>25</v>
@@ -812,7 +914,7 @@
         <v>2026</v>
       </c>
       <c r="G2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H2" t="s">
         <v>25</v>
@@ -833,7 +935,7 @@
         <v>5899998</v>
       </c>
       <c r="N2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O2" t="s">
         <v>25</v>
@@ -842,31 +944,31 @@
         <v>0</v>
       </c>
       <c r="Q2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="R2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="S2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="U2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="W2" t="s">
         <v>25</v>
       </c>
       <c r="X2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Y2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
@@ -874,13 +976,13 @@
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
         <v>25</v>
@@ -889,7 +991,7 @@
         <v>2026</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="H3" t="s">
         <v>25</v>
@@ -910,7 +1012,7 @@
         <v>5600000</v>
       </c>
       <c r="N3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="O3" t="s">
         <v>25</v>
@@ -919,31 +1021,31 @@
         <v>0</v>
       </c>
       <c r="Q3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="R3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="S3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T3" t="s">
         <v>25</v>
       </c>
       <c r="U3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="V3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="W3" t="s">
         <v>25</v>
       </c>
       <c r="X3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="Y3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
@@ -951,13 +1053,13 @@
         <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E4" t="s">
         <v>25</v>
@@ -966,7 +1068,7 @@
         <v>2026</v>
       </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="H4" t="s">
         <v>25</v>
@@ -987,7 +1089,7 @@
         <v>8800000</v>
       </c>
       <c r="N4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="O4" t="s">
         <v>25</v>
@@ -996,31 +1098,31 @@
         <v>0</v>
       </c>
       <c r="Q4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="S4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T4" t="s">
         <v>25</v>
       </c>
       <c r="U4" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="V4" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="W4" t="s">
         <v>25</v>
       </c>
       <c r="X4" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="Y4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
@@ -1028,13 +1130,13 @@
         <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E5" t="s">
         <v>25</v>
@@ -1043,7 +1145,7 @@
         <v>2026</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="H5" t="s">
         <v>25</v>
@@ -1064,7 +1166,7 @@
         <v>5599999</v>
       </c>
       <c r="N5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="O5" t="s">
         <v>25</v>
@@ -1073,31 +1175,31 @@
         <v>0</v>
       </c>
       <c r="Q5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="R5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="S5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T5" t="s">
         <v>25</v>
       </c>
       <c r="U5" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="V5" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="W5" t="s">
         <v>25</v>
       </c>
       <c r="X5" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="Y5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
@@ -1105,13 +1207,13 @@
         <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
         <v>25</v>
@@ -1120,7 +1222,7 @@
         <v>2026</v>
       </c>
       <c r="G6" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="H6" t="s">
         <v>25</v>
@@ -1141,7 +1243,7 @@
         <v>6900000</v>
       </c>
       <c r="N6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O6" t="s">
         <v>25</v>
@@ -1150,31 +1252,31 @@
         <v>0</v>
       </c>
       <c r="Q6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="R6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="S6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T6" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="U6" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="V6" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="W6" t="s">
         <v>25</v>
       </c>
       <c r="X6" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="Y6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
@@ -1182,13 +1284,13 @@
         <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="E7" t="s">
         <v>25</v>
@@ -1197,7 +1299,7 @@
         <v>2026</v>
       </c>
       <c r="G7" t="s">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="H7" t="s">
         <v>25</v>
@@ -1218,7 +1320,7 @@
         <v>3600000</v>
       </c>
       <c r="N7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O7" t="s">
         <v>25</v>
@@ -1227,31 +1329,31 @@
         <v>0</v>
       </c>
       <c r="Q7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="R7" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="S7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T7" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="U7" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="V7" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="W7" t="s">
         <v>25</v>
       </c>
       <c r="X7" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="Y7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
@@ -1259,13 +1361,13 @@
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="E8" t="s">
         <v>25</v>
@@ -1274,7 +1376,7 @@
         <v>2026</v>
       </c>
       <c r="G8" t="s">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="H8" t="s">
         <v>25</v>
@@ -1295,7 +1397,7 @@
         <v>5599999</v>
       </c>
       <c r="N8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="O8" t="s">
         <v>25</v>
@@ -1304,22 +1406,22 @@
         <v>0</v>
       </c>
       <c r="Q8" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="R8" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="S8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T8" t="s">
         <v>25</v>
       </c>
       <c r="U8" t="s">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="V8" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="W8" t="s">
         <v>25</v>
@@ -1328,7 +1430,7 @@
         <v>25</v>
       </c>
       <c r="Y8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
@@ -1336,13 +1438,13 @@
         <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="E9" t="s">
         <v>25</v>
@@ -1351,7 +1453,7 @@
         <v>2026</v>
       </c>
       <c r="G9" t="s">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="H9" t="s">
         <v>25</v>
@@ -1372,7 +1474,7 @@
         <v>6300000</v>
       </c>
       <c r="N9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O9" t="s">
         <v>25</v>
@@ -1381,31 +1483,31 @@
         <v>0</v>
       </c>
       <c r="Q9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="R9" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="S9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T9" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="U9" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="V9" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="W9" t="s">
         <v>25</v>
       </c>
       <c r="X9" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="Y9" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
@@ -1413,13 +1515,13 @@
         <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="E10" t="s">
         <v>25</v>
@@ -1428,7 +1530,7 @@
         <v>2026</v>
       </c>
       <c r="G10" t="s">
-        <v>25</v>
+        <v>87</v>
       </c>
       <c r="H10" t="s">
         <v>25</v>
@@ -1449,7 +1551,7 @@
         <v>7699999</v>
       </c>
       <c r="N10" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O10" t="s">
         <v>25</v>
@@ -1458,31 +1560,31 @@
         <v>0</v>
       </c>
       <c r="Q10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="R10" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="S10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T10" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="U10" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="V10" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="W10" t="s">
         <v>25</v>
       </c>
       <c r="X10" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="Y10" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
@@ -1490,13 +1592,13 @@
         <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="E11" t="s">
         <v>25</v>
@@ -1505,7 +1607,7 @@
         <v>2026</v>
       </c>
       <c r="G11" t="s">
-        <v>25</v>
+        <v>92</v>
       </c>
       <c r="H11" t="s">
         <v>25</v>
@@ -1526,7 +1628,7 @@
         <v>2199999</v>
       </c>
       <c r="N11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O11" t="s">
         <v>25</v>
@@ -1535,31 +1637,31 @@
         <v>0</v>
       </c>
       <c r="Q11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="R11" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="S11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T11" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="U11" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="V11" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="W11" t="s">
         <v>25</v>
       </c>
       <c r="X11" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="Y11" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
@@ -1567,13 +1669,13 @@
         <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D12" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="E12" t="s">
         <v>25</v>
@@ -1582,7 +1684,7 @@
         <v>2026</v>
       </c>
       <c r="G12" t="s">
-        <v>25</v>
+        <v>98</v>
       </c>
       <c r="H12" t="s">
         <v>25</v>
@@ -1603,7 +1705,7 @@
         <v>4799999</v>
       </c>
       <c r="N12" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O12" t="s">
         <v>25</v>
@@ -1612,31 +1714,31 @@
         <v>0</v>
       </c>
       <c r="Q12" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="R12" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="S12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T12" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="U12" t="s">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="V12" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="W12" t="s">
         <v>25</v>
       </c>
       <c r="X12" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="Y12" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
@@ -1644,13 +1746,13 @@
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="E13" t="s">
         <v>25</v>
@@ -1659,7 +1761,7 @@
         <v>2026</v>
       </c>
       <c r="G13" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="H13" t="s">
         <v>25</v>
@@ -1680,7 +1782,7 @@
         <v>5299999</v>
       </c>
       <c r="N13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O13" t="s">
         <v>25</v>
@@ -1689,31 +1791,31 @@
         <v>0</v>
       </c>
       <c r="Q13" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="R13" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="S13" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T13" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="U13" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="V13" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="W13" t="s">
         <v>25</v>
       </c>
       <c r="X13" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="Y13" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
@@ -1721,13 +1823,13 @@
         <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>107</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D14" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="E14" t="s">
         <v>25</v>
@@ -1736,7 +1838,7 @@
         <v>2026</v>
       </c>
       <c r="G14" t="s">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="H14" t="s">
         <v>25</v>
@@ -1757,7 +1859,7 @@
         <v>5399999</v>
       </c>
       <c r="N14" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O14" t="s">
         <v>25</v>
@@ -1766,31 +1868,31 @@
         <v>0</v>
       </c>
       <c r="Q14" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="R14" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="S14" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T14" t="s">
-        <v>85</v>
+        <v>111</v>
       </c>
       <c r="U14" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="V14" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="W14" t="s">
         <v>25</v>
       </c>
       <c r="X14" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="Y14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
@@ -1798,13 +1900,13 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>115</v>
       </c>
       <c r="C15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D15" t="s">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="E15" t="s">
         <v>25</v>
@@ -1813,7 +1915,7 @@
         <v>2026</v>
       </c>
       <c r="G15" t="s">
-        <v>25</v>
+        <v>117</v>
       </c>
       <c r="H15" t="s">
         <v>25</v>
@@ -1834,7 +1936,7 @@
         <v>8899999</v>
       </c>
       <c r="N15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O15" t="s">
         <v>25</v>
@@ -1843,31 +1945,31 @@
         <v>0</v>
       </c>
       <c r="Q15" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="R15" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="S15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T15" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="U15" t="s">
-        <v>91</v>
+        <v>119</v>
       </c>
       <c r="V15" t="s">
-        <v>92</v>
+        <v>120</v>
       </c>
       <c r="W15" t="s">
         <v>25</v>
       </c>
       <c r="X15" t="s">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="Y15" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
@@ -1875,13 +1977,13 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>121</v>
       </c>
       <c r="C16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D16" t="s">
-        <v>93</v>
+        <v>122</v>
       </c>
       <c r="E16" t="s">
         <v>25</v>
@@ -1890,7 +1992,7 @@
         <v>2026</v>
       </c>
       <c r="G16" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="H16" t="s">
         <v>25</v>
@@ -1911,7 +2013,7 @@
         <v>1699999</v>
       </c>
       <c r="N16" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O16" t="s">
         <v>25</v>
@@ -1920,31 +2022,31 @@
         <v>0</v>
       </c>
       <c r="Q16" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="R16" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="S16" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T16" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="U16" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="V16" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="W16" t="s">
         <v>25</v>
       </c>
       <c r="X16" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="Y16" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
@@ -1952,13 +2054,13 @@
         <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>129</v>
       </c>
       <c r="C17" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D17" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="E17" t="s">
         <v>25</v>
@@ -1967,7 +2069,7 @@
         <v>2026</v>
       </c>
       <c r="G17" t="s">
-        <v>25</v>
+        <v>131</v>
       </c>
       <c r="H17" t="s">
         <v>25</v>
@@ -1988,7 +2090,7 @@
         <v>1899999</v>
       </c>
       <c r="N17" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O17" t="s">
         <v>25</v>
@@ -1997,31 +2099,31 @@
         <v>0</v>
       </c>
       <c r="Q17" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="R17" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="S17" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T17" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="U17" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
       <c r="V17" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="W17" t="s">
         <v>25</v>
       </c>
       <c r="X17" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="Y17" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
@@ -2029,13 +2131,13 @@
         <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>134</v>
       </c>
       <c r="C18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D18" t="s">
-        <v>102</v>
+        <v>135</v>
       </c>
       <c r="E18" t="s">
         <v>25</v>
@@ -2044,7 +2146,7 @@
         <v>2026</v>
       </c>
       <c r="G18" t="s">
-        <v>25</v>
+        <v>136</v>
       </c>
       <c r="H18" t="s">
         <v>25</v>
@@ -2065,7 +2167,7 @@
         <v>2799999</v>
       </c>
       <c r="N18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O18" t="s">
         <v>25</v>
@@ -2074,35 +2176,35 @@
         <v>0</v>
       </c>
       <c r="Q18" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="R18" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="S18" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="T18" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="U18" t="s">
-        <v>103</v>
+        <v>137</v>
       </c>
       <c r="V18" t="s">
-        <v>104</v>
+        <v>138</v>
       </c>
       <c r="W18" t="s">
         <v>25</v>
       </c>
       <c r="X18" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="Y18" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update agent metadata and memory with batch 502 verification assets
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/attached_assets/cam-motors/cam-motors-inventory-import.xlsx
+++ b/attached_assets/cam-motors/cam-motors-inventory-import.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="210">
   <si>
     <t>Inventory ID</t>
   </si>
@@ -431,6 +431,219 @@
   </si>
   <si>
     <t>https://cammotors.gy/api/storage/objects/20f063af-0030-4d7c-b81f-d345f67a918c, https://cammotors.gy/api/storage/objects/4d22f9ec-9a99-4476-822d-32c5939a2e3a, https://cammotors.gy/api/storage/objects/0d631b89-aa5c-4785-b260-011faa94f3d4, https://cammotors.gy/api/storage/objects/ce3d5a52-8267-4cd4-baf2-f3b0da46033b, https://cammotors.gy/api/storage/objects/d44b4085-dee6-43d7-bf67-d16ddd04ee37, https://cammotors.gy/api/storage/objects/0f60f619-73a2-42f6-8a36-426de7d040b0, https://cammotors.gy/api/storage/objects/17cee22d-6846-4aaa-b5ee-e80aff10fa17, https://cammotors.gy/api/storage/objects/000f256e-0223-4dd3-a73c-c13d93051840, https://cammotors.gy/api/storage/objects/ca0a4043-a879-4f09-85eb-9d7a70f4cf96, https://cammotors.gy/api/storage/objects/39b3f343-cd8c-416d-897d-438e27a5480f, https://cammotors.gy/api/storage/objects/97e00770-0fcb-446b-b14d-103aebdc9845, https://cammotors.gy/api/storage/objects/03a582ef-19a9-42cb-85eb-e4d439e97087, https://cammotors.gy/api/storage/objects/ba6549db-7d20-4ab4-9455-6b054c9a27f7, https://cammotors.gy/api/storage/objects/8f815e28-1fee-4b10-bb33-ed81da97a21f</t>
+  </si>
+  <si>
+    <t>LVC105YYDGJR6Z82K</t>
+  </si>
+  <si>
+    <t>ENV3KCBURFYXJJAYA</t>
+  </si>
+  <si>
+    <t>LVCUPEYJ32MCZ4W38</t>
+  </si>
+  <si>
+    <t>ENVDRWZNDZG306SXD</t>
+  </si>
+  <si>
+    <t>L1C86ARAYKW4KX7WX</t>
+  </si>
+  <si>
+    <t>ENPBC4MN0V9A2RRCA</t>
+  </si>
+  <si>
+    <t>white</t>
+  </si>
+  <si>
+    <t>L1CBCUA5GAHH0H8ZU</t>
+  </si>
+  <si>
+    <t>ENDD9MA9XKFJBL8Z2</t>
+  </si>
+  <si>
+    <t>Shadow Grey</t>
+  </si>
+  <si>
+    <t>L1C3G52EY3GSEXRB1</t>
+  </si>
+  <si>
+    <t>ENGAM8N7HKZ0103MW</t>
+  </si>
+  <si>
+    <t>L1C4YN7LHZWDNG3U5</t>
+  </si>
+  <si>
+    <t>EN44564DSTFYTKC9K</t>
+  </si>
+  <si>
+    <t>Silver</t>
+  </si>
+  <si>
+    <t>L1CM40CHKLZBVUW7A</t>
+  </si>
+  <si>
+    <t>EN6XBSSG5ZT6H5PPZ</t>
+  </si>
+  <si>
+    <t>L1CP33LMJ6YMAVMGF</t>
+  </si>
+  <si>
+    <t>EN69XMRJVDM55VF5G</t>
+  </si>
+  <si>
+    <t>LVCX0FC4JEBAW0B3M</t>
+  </si>
+  <si>
+    <t>ENFD01VUC1NAVA9YL</t>
+  </si>
+  <si>
+    <t>LVCRGKGHZR59Z52JL</t>
+  </si>
+  <si>
+    <t>ENW6PUR8TP2A4SGKC</t>
+  </si>
+  <si>
+    <t>LVC8NC4FW12GRFDWU</t>
+  </si>
+  <si>
+    <t>ENKGWGXAU0RB4ABCG</t>
+  </si>
+  <si>
+    <t>LVC5HJVPDL8BUAEDL</t>
+  </si>
+  <si>
+    <t>EN9KD2GGWHSLVPKUJ</t>
+  </si>
+  <si>
+    <t>L1CDFPK9AGWY5653T</t>
+  </si>
+  <si>
+    <t>ENJYMFUAF172FS821</t>
+  </si>
+  <si>
+    <t>L1CDVBW27T47EU2B1</t>
+  </si>
+  <si>
+    <t>ENY6KD5118173TTCX</t>
+  </si>
+  <si>
+    <t>LVCKY5NYZAW3C79UN</t>
+  </si>
+  <si>
+    <t>EN8YGVRMC5HNXBFES</t>
+  </si>
+  <si>
+    <t>LVCEKL760APPK5APX</t>
+  </si>
+  <si>
+    <t>EN8FWLVUYY1YJK08S</t>
+  </si>
+  <si>
+    <t>LVCRYS888001XDF1C</t>
+  </si>
+  <si>
+    <t>ENL0LFAGCJNUHWEMR</t>
+  </si>
+  <si>
+    <t>LVCS6M4BM4UGCYGEY</t>
+  </si>
+  <si>
+    <t>ENS65Z6C5GX0EPHNC</t>
+  </si>
+  <si>
+    <t>LVCNM3B1RT4GCHA4F</t>
+  </si>
+  <si>
+    <t>ENAXX9919AYSGUNS8</t>
+  </si>
+  <si>
+    <t>LVCUER9W1Y596A4EM</t>
+  </si>
+  <si>
+    <t>ENGH4V25LM3ER991A</t>
+  </si>
+  <si>
+    <t>LVC7EMKFBZ1WBPXLX</t>
+  </si>
+  <si>
+    <t>ENRCGEF0FX41NDKYP</t>
+  </si>
+  <si>
+    <t>LVCZDRJJ3YFXP4C11</t>
+  </si>
+  <si>
+    <t>EN3C2845DC6S1ZAYR</t>
+  </si>
+  <si>
+    <t>LVCXE0J6GS4CLZ4ZZ</t>
+  </si>
+  <si>
+    <t>EN7KJ8TMS01CF09ZN</t>
+  </si>
+  <si>
+    <t>LVCRFCM9GY1WRGHAS</t>
+  </si>
+  <si>
+    <t>EN7W1VYNAPGDWXXAC</t>
+  </si>
+  <si>
+    <t>LVCSW8B3YGA6HKVGA</t>
+  </si>
+  <si>
+    <t>ENNJLU26DH2XD25CH</t>
+  </si>
+  <si>
+    <t>LVCLZ1XNKPDU6BLWZ</t>
+  </si>
+  <si>
+    <t>EN8LNDSSLAY3D4XCM</t>
+  </si>
+  <si>
+    <t>LVC4C01CMFYM9KJPM</t>
+  </si>
+  <si>
+    <t>ENHW1XPVGBCUBA55C</t>
+  </si>
+  <si>
+    <t>LVCRZVCRKMVJL29AC</t>
+  </si>
+  <si>
+    <t>ENRJTJ2HUJ4FC3PD8</t>
+  </si>
+  <si>
+    <t>LVC9EKSUGPJ8E3BTC</t>
+  </si>
+  <si>
+    <t>EN9YHAZ0F4H1SKEWU</t>
+  </si>
+  <si>
+    <t>LVCJWVR5FZFHK06HB</t>
+  </si>
+  <si>
+    <t>ENR31DLT21ED3TH6P</t>
+  </si>
+  <si>
+    <t>LVCNU7M4DELCM6ZNB</t>
+  </si>
+  <si>
+    <t>ENEAEPJVSBKVJRS51</t>
+  </si>
+  <si>
+    <t>LVCAZP9VLAA3ZE0VL</t>
+  </si>
+  <si>
+    <t>EN9ZLAXVPDN1G1DMH</t>
+  </si>
+  <si>
+    <t>LVC0FRS0PZHAHSE7J</t>
+  </si>
+  <si>
+    <t>ENDMCVPZS79H6JY3F</t>
+  </si>
+  <si>
+    <t>LVCPPT64W79HSP57G</t>
+  </si>
+  <si>
+    <t>ENSE8ZYABX4K3CSSH</t>
   </si>
 </sst>
 </file>
@@ -811,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y18"/>
+  <dimension ref="A1:Y52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="25" width="18" customWidth="1"/>
@@ -2203,6 +2416,2624 @@
         <v>46</v>
       </c>
     </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" t="s">
+        <v>139</v>
+      </c>
+      <c r="C19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F19">
+        <v>2026</v>
+      </c>
+      <c r="G19" t="s">
+        <v>140</v>
+      </c>
+      <c r="H19" t="s">
+        <v>25</v>
+      </c>
+      <c r="I19" t="s">
+        <v>25</v>
+      </c>
+      <c r="J19" t="s">
+        <v>25</v>
+      </c>
+      <c r="K19" t="s">
+        <v>25</v>
+      </c>
+      <c r="L19">
+        <v>7900000</v>
+      </c>
+      <c r="M19">
+        <v>5899998</v>
+      </c>
+      <c r="N19" t="s">
+        <v>30</v>
+      </c>
+      <c r="O19" t="s">
+        <v>25</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>31</v>
+      </c>
+      <c r="R19" t="s">
+        <v>32</v>
+      </c>
+      <c r="S19" t="s">
+        <v>33</v>
+      </c>
+      <c r="T19" t="s">
+        <v>28</v>
+      </c>
+      <c r="U19" t="s">
+        <v>34</v>
+      </c>
+      <c r="V19" t="s">
+        <v>34</v>
+      </c>
+      <c r="W19" t="s">
+        <v>25</v>
+      </c>
+      <c r="X19" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>141</v>
+      </c>
+      <c r="C20" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20">
+        <v>2026</v>
+      </c>
+      <c r="G20" t="s">
+        <v>142</v>
+      </c>
+      <c r="H20" t="s">
+        <v>25</v>
+      </c>
+      <c r="I20" t="s">
+        <v>25</v>
+      </c>
+      <c r="J20" t="s">
+        <v>25</v>
+      </c>
+      <c r="K20" t="s">
+        <v>25</v>
+      </c>
+      <c r="L20">
+        <v>7900000</v>
+      </c>
+      <c r="M20">
+        <v>5899998</v>
+      </c>
+      <c r="N20" t="s">
+        <v>30</v>
+      </c>
+      <c r="O20" t="s">
+        <v>25</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>31</v>
+      </c>
+      <c r="R20" t="s">
+        <v>32</v>
+      </c>
+      <c r="S20" t="s">
+        <v>33</v>
+      </c>
+      <c r="T20" t="s">
+        <v>28</v>
+      </c>
+      <c r="U20" t="s">
+        <v>34</v>
+      </c>
+      <c r="V20" t="s">
+        <v>34</v>
+      </c>
+      <c r="W20" t="s">
+        <v>25</v>
+      </c>
+      <c r="X20" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
+        <v>143</v>
+      </c>
+      <c r="C21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21">
+        <v>2026</v>
+      </c>
+      <c r="G21" t="s">
+        <v>144</v>
+      </c>
+      <c r="H21" t="s">
+        <v>25</v>
+      </c>
+      <c r="I21" t="s">
+        <v>25</v>
+      </c>
+      <c r="J21" t="s">
+        <v>25</v>
+      </c>
+      <c r="K21" t="s">
+        <v>25</v>
+      </c>
+      <c r="L21">
+        <v>6990000</v>
+      </c>
+      <c r="M21">
+        <v>5600000</v>
+      </c>
+      <c r="N21" t="s">
+        <v>41</v>
+      </c>
+      <c r="O21" t="s">
+        <v>25</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>145</v>
+      </c>
+      <c r="R21" t="s">
+        <v>42</v>
+      </c>
+      <c r="S21" t="s">
+        <v>33</v>
+      </c>
+      <c r="T21" t="s">
+        <v>25</v>
+      </c>
+      <c r="U21" t="s">
+        <v>43</v>
+      </c>
+      <c r="V21" t="s">
+        <v>44</v>
+      </c>
+      <c r="W21" t="s">
+        <v>25</v>
+      </c>
+      <c r="X21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" t="s">
+        <v>146</v>
+      </c>
+      <c r="C22" t="s">
+        <v>38</v>
+      </c>
+      <c r="D22" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22">
+        <v>2026</v>
+      </c>
+      <c r="G22" t="s">
+        <v>147</v>
+      </c>
+      <c r="H22" t="s">
+        <v>25</v>
+      </c>
+      <c r="I22" t="s">
+        <v>25</v>
+      </c>
+      <c r="J22" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22" t="s">
+        <v>25</v>
+      </c>
+      <c r="L22">
+        <v>6990000</v>
+      </c>
+      <c r="M22">
+        <v>5600000</v>
+      </c>
+      <c r="N22" t="s">
+        <v>41</v>
+      </c>
+      <c r="O22" t="s">
+        <v>25</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>148</v>
+      </c>
+      <c r="R22" t="s">
+        <v>42</v>
+      </c>
+      <c r="S22" t="s">
+        <v>33</v>
+      </c>
+      <c r="T22" t="s">
+        <v>25</v>
+      </c>
+      <c r="U22" t="s">
+        <v>43</v>
+      </c>
+      <c r="V22" t="s">
+        <v>44</v>
+      </c>
+      <c r="W22" t="s">
+        <v>25</v>
+      </c>
+      <c r="X22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s">
+        <v>149</v>
+      </c>
+      <c r="C23" t="s">
+        <v>38</v>
+      </c>
+      <c r="D23" t="s">
+        <v>48</v>
+      </c>
+      <c r="E23" t="s">
+        <v>25</v>
+      </c>
+      <c r="F23">
+        <v>2026</v>
+      </c>
+      <c r="G23" t="s">
+        <v>150</v>
+      </c>
+      <c r="H23" t="s">
+        <v>25</v>
+      </c>
+      <c r="I23" t="s">
+        <v>25</v>
+      </c>
+      <c r="J23" t="s">
+        <v>25</v>
+      </c>
+      <c r="K23" t="s">
+        <v>25</v>
+      </c>
+      <c r="L23">
+        <v>11500000</v>
+      </c>
+      <c r="M23">
+        <v>8800000</v>
+      </c>
+      <c r="N23" t="s">
+        <v>41</v>
+      </c>
+      <c r="O23" t="s">
+        <v>25</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>76</v>
+      </c>
+      <c r="R23" t="s">
+        <v>42</v>
+      </c>
+      <c r="S23" t="s">
+        <v>33</v>
+      </c>
+      <c r="T23" t="s">
+        <v>25</v>
+      </c>
+      <c r="U23" t="s">
+        <v>50</v>
+      </c>
+      <c r="V23" t="s">
+        <v>51</v>
+      </c>
+      <c r="W23" t="s">
+        <v>25</v>
+      </c>
+      <c r="X23" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" t="s">
+        <v>151</v>
+      </c>
+      <c r="C24" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24">
+        <v>2026</v>
+      </c>
+      <c r="G24" t="s">
+        <v>152</v>
+      </c>
+      <c r="H24" t="s">
+        <v>25</v>
+      </c>
+      <c r="I24" t="s">
+        <v>25</v>
+      </c>
+      <c r="J24" t="s">
+        <v>25</v>
+      </c>
+      <c r="K24" t="s">
+        <v>25</v>
+      </c>
+      <c r="L24">
+        <v>11500000</v>
+      </c>
+      <c r="M24">
+        <v>8800000</v>
+      </c>
+      <c r="N24" t="s">
+        <v>41</v>
+      </c>
+      <c r="O24" t="s">
+        <v>25</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>153</v>
+      </c>
+      <c r="R24" t="s">
+        <v>42</v>
+      </c>
+      <c r="S24" t="s">
+        <v>33</v>
+      </c>
+      <c r="T24" t="s">
+        <v>25</v>
+      </c>
+      <c r="U24" t="s">
+        <v>50</v>
+      </c>
+      <c r="V24" t="s">
+        <v>51</v>
+      </c>
+      <c r="W24" t="s">
+        <v>25</v>
+      </c>
+      <c r="X24" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" t="s">
+        <v>154</v>
+      </c>
+      <c r="C25" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25" t="s">
+        <v>54</v>
+      </c>
+      <c r="E25" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25">
+        <v>2026</v>
+      </c>
+      <c r="G25" t="s">
+        <v>155</v>
+      </c>
+      <c r="H25" t="s">
+        <v>25</v>
+      </c>
+      <c r="I25" t="s">
+        <v>25</v>
+      </c>
+      <c r="J25" t="s">
+        <v>25</v>
+      </c>
+      <c r="K25" t="s">
+        <v>25</v>
+      </c>
+      <c r="L25">
+        <v>6990000</v>
+      </c>
+      <c r="M25">
+        <v>5599999</v>
+      </c>
+      <c r="N25" t="s">
+        <v>41</v>
+      </c>
+      <c r="O25" t="s">
+        <v>25</v>
+      </c>
+      <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>145</v>
+      </c>
+      <c r="R25" t="s">
+        <v>42</v>
+      </c>
+      <c r="S25" t="s">
+        <v>33</v>
+      </c>
+      <c r="T25" t="s">
+        <v>25</v>
+      </c>
+      <c r="U25" t="s">
+        <v>56</v>
+      </c>
+      <c r="V25" t="s">
+        <v>57</v>
+      </c>
+      <c r="W25" t="s">
+        <v>25</v>
+      </c>
+      <c r="X25" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>156</v>
+      </c>
+      <c r="C26" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" t="s">
+        <v>54</v>
+      </c>
+      <c r="E26" t="s">
+        <v>25</v>
+      </c>
+      <c r="F26">
+        <v>2026</v>
+      </c>
+      <c r="G26" t="s">
+        <v>157</v>
+      </c>
+      <c r="H26" t="s">
+        <v>25</v>
+      </c>
+      <c r="I26" t="s">
+        <v>25</v>
+      </c>
+      <c r="J26" t="s">
+        <v>25</v>
+      </c>
+      <c r="K26" t="s">
+        <v>25</v>
+      </c>
+      <c r="L26">
+        <v>6990000</v>
+      </c>
+      <c r="M26">
+        <v>5599999</v>
+      </c>
+      <c r="N26" t="s">
+        <v>41</v>
+      </c>
+      <c r="O26" t="s">
+        <v>25</v>
+      </c>
+      <c r="P26">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>153</v>
+      </c>
+      <c r="R26" t="s">
+        <v>42</v>
+      </c>
+      <c r="S26" t="s">
+        <v>33</v>
+      </c>
+      <c r="T26" t="s">
+        <v>25</v>
+      </c>
+      <c r="U26" t="s">
+        <v>56</v>
+      </c>
+      <c r="V26" t="s">
+        <v>57</v>
+      </c>
+      <c r="W26" t="s">
+        <v>25</v>
+      </c>
+      <c r="X26" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>158</v>
+      </c>
+      <c r="C27" t="s">
+        <v>27</v>
+      </c>
+      <c r="D27" t="s">
+        <v>60</v>
+      </c>
+      <c r="E27" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27">
+        <v>2026</v>
+      </c>
+      <c r="G27" t="s">
+        <v>159</v>
+      </c>
+      <c r="H27" t="s">
+        <v>25</v>
+      </c>
+      <c r="I27" t="s">
+        <v>25</v>
+      </c>
+      <c r="J27" t="s">
+        <v>25</v>
+      </c>
+      <c r="K27" t="s">
+        <v>25</v>
+      </c>
+      <c r="L27">
+        <v>8899999</v>
+      </c>
+      <c r="M27">
+        <v>6900000</v>
+      </c>
+      <c r="N27" t="s">
+        <v>30</v>
+      </c>
+      <c r="O27" t="s">
+        <v>25</v>
+      </c>
+      <c r="P27">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>31</v>
+      </c>
+      <c r="R27" t="s">
+        <v>32</v>
+      </c>
+      <c r="S27" t="s">
+        <v>33</v>
+      </c>
+      <c r="T27" t="s">
+        <v>60</v>
+      </c>
+      <c r="U27" t="s">
+        <v>62</v>
+      </c>
+      <c r="V27" t="s">
+        <v>63</v>
+      </c>
+      <c r="W27" t="s">
+        <v>25</v>
+      </c>
+      <c r="X27" t="s">
+        <v>64</v>
+      </c>
+      <c r="Y27" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" t="s">
+        <v>160</v>
+      </c>
+      <c r="C28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" t="s">
+        <v>60</v>
+      </c>
+      <c r="E28" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28">
+        <v>2026</v>
+      </c>
+      <c r="G28" t="s">
+        <v>161</v>
+      </c>
+      <c r="H28" t="s">
+        <v>25</v>
+      </c>
+      <c r="I28" t="s">
+        <v>25</v>
+      </c>
+      <c r="J28" t="s">
+        <v>25</v>
+      </c>
+      <c r="K28" t="s">
+        <v>25</v>
+      </c>
+      <c r="L28">
+        <v>8899999</v>
+      </c>
+      <c r="M28">
+        <v>6900000</v>
+      </c>
+      <c r="N28" t="s">
+        <v>30</v>
+      </c>
+      <c r="O28" t="s">
+        <v>25</v>
+      </c>
+      <c r="P28">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>31</v>
+      </c>
+      <c r="R28" t="s">
+        <v>32</v>
+      </c>
+      <c r="S28" t="s">
+        <v>33</v>
+      </c>
+      <c r="T28" t="s">
+        <v>60</v>
+      </c>
+      <c r="U28" t="s">
+        <v>62</v>
+      </c>
+      <c r="V28" t="s">
+        <v>63</v>
+      </c>
+      <c r="W28" t="s">
+        <v>25</v>
+      </c>
+      <c r="X28" t="s">
+        <v>64</v>
+      </c>
+      <c r="Y28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" t="s">
+        <v>162</v>
+      </c>
+      <c r="C29" t="s">
+        <v>27</v>
+      </c>
+      <c r="D29" t="s">
+        <v>66</v>
+      </c>
+      <c r="E29" t="s">
+        <v>25</v>
+      </c>
+      <c r="F29">
+        <v>2026</v>
+      </c>
+      <c r="G29" t="s">
+        <v>163</v>
+      </c>
+      <c r="H29" t="s">
+        <v>25</v>
+      </c>
+      <c r="I29" t="s">
+        <v>25</v>
+      </c>
+      <c r="J29" t="s">
+        <v>25</v>
+      </c>
+      <c r="K29" t="s">
+        <v>25</v>
+      </c>
+      <c r="L29">
+        <v>5600000</v>
+      </c>
+      <c r="M29">
+        <v>3600000</v>
+      </c>
+      <c r="N29" t="s">
+        <v>30</v>
+      </c>
+      <c r="O29" t="s">
+        <v>25</v>
+      </c>
+      <c r="P29">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>31</v>
+      </c>
+      <c r="R29" t="s">
+        <v>68</v>
+      </c>
+      <c r="S29" t="s">
+        <v>33</v>
+      </c>
+      <c r="T29" t="s">
+        <v>69</v>
+      </c>
+      <c r="U29" t="s">
+        <v>70</v>
+      </c>
+      <c r="V29" t="s">
+        <v>71</v>
+      </c>
+      <c r="W29" t="s">
+        <v>25</v>
+      </c>
+      <c r="X29" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y29" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" t="s">
+        <v>164</v>
+      </c>
+      <c r="C30" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" t="s">
+        <v>66</v>
+      </c>
+      <c r="E30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F30">
+        <v>2026</v>
+      </c>
+      <c r="G30" t="s">
+        <v>165</v>
+      </c>
+      <c r="H30" t="s">
+        <v>25</v>
+      </c>
+      <c r="I30" t="s">
+        <v>25</v>
+      </c>
+      <c r="J30" t="s">
+        <v>25</v>
+      </c>
+      <c r="K30" t="s">
+        <v>25</v>
+      </c>
+      <c r="L30">
+        <v>5600000</v>
+      </c>
+      <c r="M30">
+        <v>3600000</v>
+      </c>
+      <c r="N30" t="s">
+        <v>30</v>
+      </c>
+      <c r="O30" t="s">
+        <v>25</v>
+      </c>
+      <c r="P30">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>31</v>
+      </c>
+      <c r="R30" t="s">
+        <v>68</v>
+      </c>
+      <c r="S30" t="s">
+        <v>33</v>
+      </c>
+      <c r="T30" t="s">
+        <v>69</v>
+      </c>
+      <c r="U30" t="s">
+        <v>70</v>
+      </c>
+      <c r="V30" t="s">
+        <v>71</v>
+      </c>
+      <c r="W30" t="s">
+        <v>25</v>
+      </c>
+      <c r="X30" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y30" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31" t="s">
+        <v>166</v>
+      </c>
+      <c r="C31" t="s">
+        <v>38</v>
+      </c>
+      <c r="D31" t="s">
+        <v>74</v>
+      </c>
+      <c r="E31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F31">
+        <v>2026</v>
+      </c>
+      <c r="G31" t="s">
+        <v>167</v>
+      </c>
+      <c r="H31" t="s">
+        <v>25</v>
+      </c>
+      <c r="I31" t="s">
+        <v>25</v>
+      </c>
+      <c r="J31" t="s">
+        <v>25</v>
+      </c>
+      <c r="K31" t="s">
+        <v>25</v>
+      </c>
+      <c r="L31">
+        <v>6990000</v>
+      </c>
+      <c r="M31">
+        <v>5599999</v>
+      </c>
+      <c r="N31" t="s">
+        <v>41</v>
+      </c>
+      <c r="O31" t="s">
+        <v>25</v>
+      </c>
+      <c r="P31">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>76</v>
+      </c>
+      <c r="R31" t="s">
+        <v>42</v>
+      </c>
+      <c r="S31" t="s">
+        <v>33</v>
+      </c>
+      <c r="T31" t="s">
+        <v>25</v>
+      </c>
+      <c r="U31" t="s">
+        <v>77</v>
+      </c>
+      <c r="V31" t="s">
+        <v>78</v>
+      </c>
+      <c r="W31" t="s">
+        <v>25</v>
+      </c>
+      <c r="X31" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32" t="s">
+        <v>168</v>
+      </c>
+      <c r="C32" t="s">
+        <v>38</v>
+      </c>
+      <c r="D32" t="s">
+        <v>74</v>
+      </c>
+      <c r="E32" t="s">
+        <v>25</v>
+      </c>
+      <c r="F32">
+        <v>2026</v>
+      </c>
+      <c r="G32" t="s">
+        <v>169</v>
+      </c>
+      <c r="H32" t="s">
+        <v>25</v>
+      </c>
+      <c r="I32" t="s">
+        <v>25</v>
+      </c>
+      <c r="J32" t="s">
+        <v>25</v>
+      </c>
+      <c r="K32" t="s">
+        <v>25</v>
+      </c>
+      <c r="L32">
+        <v>6990000</v>
+      </c>
+      <c r="M32">
+        <v>5599999</v>
+      </c>
+      <c r="N32" t="s">
+        <v>41</v>
+      </c>
+      <c r="O32" t="s">
+        <v>25</v>
+      </c>
+      <c r="P32">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>76</v>
+      </c>
+      <c r="R32" t="s">
+        <v>42</v>
+      </c>
+      <c r="S32" t="s">
+        <v>33</v>
+      </c>
+      <c r="T32" t="s">
+        <v>25</v>
+      </c>
+      <c r="U32" t="s">
+        <v>77</v>
+      </c>
+      <c r="V32" t="s">
+        <v>78</v>
+      </c>
+      <c r="W32" t="s">
+        <v>25</v>
+      </c>
+      <c r="X32" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33" t="s">
+        <v>170</v>
+      </c>
+      <c r="C33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" t="s">
+        <v>80</v>
+      </c>
+      <c r="E33" t="s">
+        <v>25</v>
+      </c>
+      <c r="F33">
+        <v>2026</v>
+      </c>
+      <c r="G33" t="s">
+        <v>171</v>
+      </c>
+      <c r="H33" t="s">
+        <v>25</v>
+      </c>
+      <c r="I33" t="s">
+        <v>25</v>
+      </c>
+      <c r="J33" t="s">
+        <v>25</v>
+      </c>
+      <c r="K33" t="s">
+        <v>25</v>
+      </c>
+      <c r="L33">
+        <v>8299998</v>
+      </c>
+      <c r="M33">
+        <v>6300000</v>
+      </c>
+      <c r="N33" t="s">
+        <v>30</v>
+      </c>
+      <c r="O33" t="s">
+        <v>25</v>
+      </c>
+      <c r="P33">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>31</v>
+      </c>
+      <c r="R33" t="s">
+        <v>68</v>
+      </c>
+      <c r="S33" t="s">
+        <v>33</v>
+      </c>
+      <c r="T33" t="s">
+        <v>69</v>
+      </c>
+      <c r="U33" t="s">
+        <v>82</v>
+      </c>
+      <c r="V33" t="s">
+        <v>83</v>
+      </c>
+      <c r="W33" t="s">
+        <v>25</v>
+      </c>
+      <c r="X33" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>25</v>
+      </c>
+      <c r="B34" t="s">
+        <v>172</v>
+      </c>
+      <c r="C34" t="s">
+        <v>27</v>
+      </c>
+      <c r="D34" t="s">
+        <v>80</v>
+      </c>
+      <c r="E34" t="s">
+        <v>25</v>
+      </c>
+      <c r="F34">
+        <v>2026</v>
+      </c>
+      <c r="G34" t="s">
+        <v>173</v>
+      </c>
+      <c r="H34" t="s">
+        <v>25</v>
+      </c>
+      <c r="I34" t="s">
+        <v>25</v>
+      </c>
+      <c r="J34" t="s">
+        <v>25</v>
+      </c>
+      <c r="K34" t="s">
+        <v>25</v>
+      </c>
+      <c r="L34">
+        <v>8299998</v>
+      </c>
+      <c r="M34">
+        <v>6300000</v>
+      </c>
+      <c r="N34" t="s">
+        <v>30</v>
+      </c>
+      <c r="O34" t="s">
+        <v>25</v>
+      </c>
+      <c r="P34">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>31</v>
+      </c>
+      <c r="R34" t="s">
+        <v>68</v>
+      </c>
+      <c r="S34" t="s">
+        <v>33</v>
+      </c>
+      <c r="T34" t="s">
+        <v>69</v>
+      </c>
+      <c r="U34" t="s">
+        <v>82</v>
+      </c>
+      <c r="V34" t="s">
+        <v>83</v>
+      </c>
+      <c r="W34" t="s">
+        <v>25</v>
+      </c>
+      <c r="X34" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y34" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>25</v>
+      </c>
+      <c r="B35" t="s">
+        <v>174</v>
+      </c>
+      <c r="C35" t="s">
+        <v>27</v>
+      </c>
+      <c r="D35" t="s">
+        <v>86</v>
+      </c>
+      <c r="E35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F35">
+        <v>2026</v>
+      </c>
+      <c r="G35" t="s">
+        <v>175</v>
+      </c>
+      <c r="H35" t="s">
+        <v>25</v>
+      </c>
+      <c r="I35" t="s">
+        <v>25</v>
+      </c>
+      <c r="J35" t="s">
+        <v>25</v>
+      </c>
+      <c r="K35" t="s">
+        <v>25</v>
+      </c>
+      <c r="L35">
+        <v>9700000</v>
+      </c>
+      <c r="M35">
+        <v>7699999</v>
+      </c>
+      <c r="N35" t="s">
+        <v>30</v>
+      </c>
+      <c r="O35" t="s">
+        <v>25</v>
+      </c>
+      <c r="P35">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>31</v>
+      </c>
+      <c r="R35" t="s">
+        <v>68</v>
+      </c>
+      <c r="S35" t="s">
+        <v>33</v>
+      </c>
+      <c r="T35" t="s">
+        <v>69</v>
+      </c>
+      <c r="U35" t="s">
+        <v>88</v>
+      </c>
+      <c r="V35" t="s">
+        <v>89</v>
+      </c>
+      <c r="W35" t="s">
+        <v>25</v>
+      </c>
+      <c r="X35" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y35" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B36" t="s">
+        <v>176</v>
+      </c>
+      <c r="C36" t="s">
+        <v>27</v>
+      </c>
+      <c r="D36" t="s">
+        <v>86</v>
+      </c>
+      <c r="E36" t="s">
+        <v>25</v>
+      </c>
+      <c r="F36">
+        <v>2026</v>
+      </c>
+      <c r="G36" t="s">
+        <v>177</v>
+      </c>
+      <c r="H36" t="s">
+        <v>25</v>
+      </c>
+      <c r="I36" t="s">
+        <v>25</v>
+      </c>
+      <c r="J36" t="s">
+        <v>25</v>
+      </c>
+      <c r="K36" t="s">
+        <v>25</v>
+      </c>
+      <c r="L36">
+        <v>9700000</v>
+      </c>
+      <c r="M36">
+        <v>7699999</v>
+      </c>
+      <c r="N36" t="s">
+        <v>30</v>
+      </c>
+      <c r="O36" t="s">
+        <v>25</v>
+      </c>
+      <c r="P36">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>31</v>
+      </c>
+      <c r="R36" t="s">
+        <v>68</v>
+      </c>
+      <c r="S36" t="s">
+        <v>33</v>
+      </c>
+      <c r="T36" t="s">
+        <v>69</v>
+      </c>
+      <c r="U36" t="s">
+        <v>88</v>
+      </c>
+      <c r="V36" t="s">
+        <v>89</v>
+      </c>
+      <c r="W36" t="s">
+        <v>25</v>
+      </c>
+      <c r="X36" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y36" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B37" t="s">
+        <v>178</v>
+      </c>
+      <c r="C37" t="s">
+        <v>27</v>
+      </c>
+      <c r="D37" t="s">
+        <v>91</v>
+      </c>
+      <c r="E37" t="s">
+        <v>25</v>
+      </c>
+      <c r="F37">
+        <v>2026</v>
+      </c>
+      <c r="G37" t="s">
+        <v>179</v>
+      </c>
+      <c r="H37" t="s">
+        <v>25</v>
+      </c>
+      <c r="I37" t="s">
+        <v>25</v>
+      </c>
+      <c r="J37" t="s">
+        <v>25</v>
+      </c>
+      <c r="K37" t="s">
+        <v>25</v>
+      </c>
+      <c r="L37">
+        <v>4200000</v>
+      </c>
+      <c r="M37">
+        <v>2199999</v>
+      </c>
+      <c r="N37" t="s">
+        <v>30</v>
+      </c>
+      <c r="O37" t="s">
+        <v>25</v>
+      </c>
+      <c r="P37">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>31</v>
+      </c>
+      <c r="R37" t="s">
+        <v>68</v>
+      </c>
+      <c r="S37" t="s">
+        <v>33</v>
+      </c>
+      <c r="T37" t="s">
+        <v>69</v>
+      </c>
+      <c r="U37" t="s">
+        <v>93</v>
+      </c>
+      <c r="V37" t="s">
+        <v>94</v>
+      </c>
+      <c r="W37" t="s">
+        <v>25</v>
+      </c>
+      <c r="X37" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y37" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>25</v>
+      </c>
+      <c r="B38" t="s">
+        <v>180</v>
+      </c>
+      <c r="C38" t="s">
+        <v>27</v>
+      </c>
+      <c r="D38" t="s">
+        <v>91</v>
+      </c>
+      <c r="E38" t="s">
+        <v>25</v>
+      </c>
+      <c r="F38">
+        <v>2026</v>
+      </c>
+      <c r="G38" t="s">
+        <v>181</v>
+      </c>
+      <c r="H38" t="s">
+        <v>25</v>
+      </c>
+      <c r="I38" t="s">
+        <v>25</v>
+      </c>
+      <c r="J38" t="s">
+        <v>25</v>
+      </c>
+      <c r="K38" t="s">
+        <v>25</v>
+      </c>
+      <c r="L38">
+        <v>4200000</v>
+      </c>
+      <c r="M38">
+        <v>2199999</v>
+      </c>
+      <c r="N38" t="s">
+        <v>30</v>
+      </c>
+      <c r="O38" t="s">
+        <v>25</v>
+      </c>
+      <c r="P38">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>31</v>
+      </c>
+      <c r="R38" t="s">
+        <v>68</v>
+      </c>
+      <c r="S38" t="s">
+        <v>33</v>
+      </c>
+      <c r="T38" t="s">
+        <v>69</v>
+      </c>
+      <c r="U38" t="s">
+        <v>93</v>
+      </c>
+      <c r="V38" t="s">
+        <v>94</v>
+      </c>
+      <c r="W38" t="s">
+        <v>25</v>
+      </c>
+      <c r="X38" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y38" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>25</v>
+      </c>
+      <c r="B39" t="s">
+        <v>182</v>
+      </c>
+      <c r="C39" t="s">
+        <v>27</v>
+      </c>
+      <c r="D39" t="s">
+        <v>97</v>
+      </c>
+      <c r="E39" t="s">
+        <v>25</v>
+      </c>
+      <c r="F39">
+        <v>2026</v>
+      </c>
+      <c r="G39" t="s">
+        <v>183</v>
+      </c>
+      <c r="H39" t="s">
+        <v>25</v>
+      </c>
+      <c r="I39" t="s">
+        <v>25</v>
+      </c>
+      <c r="J39" t="s">
+        <v>25</v>
+      </c>
+      <c r="K39" t="s">
+        <v>25</v>
+      </c>
+      <c r="L39">
+        <v>6799999</v>
+      </c>
+      <c r="M39">
+        <v>4799999</v>
+      </c>
+      <c r="N39" t="s">
+        <v>30</v>
+      </c>
+      <c r="O39" t="s">
+        <v>25</v>
+      </c>
+      <c r="P39">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>76</v>
+      </c>
+      <c r="R39" t="s">
+        <v>68</v>
+      </c>
+      <c r="S39" t="s">
+        <v>33</v>
+      </c>
+      <c r="T39" t="s">
+        <v>99</v>
+      </c>
+      <c r="U39" t="s">
+        <v>100</v>
+      </c>
+      <c r="V39" t="s">
+        <v>101</v>
+      </c>
+      <c r="W39" t="s">
+        <v>25</v>
+      </c>
+      <c r="X39" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y39" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>25</v>
+      </c>
+      <c r="B40" t="s">
+        <v>184</v>
+      </c>
+      <c r="C40" t="s">
+        <v>27</v>
+      </c>
+      <c r="D40" t="s">
+        <v>97</v>
+      </c>
+      <c r="E40" t="s">
+        <v>25</v>
+      </c>
+      <c r="F40">
+        <v>2026</v>
+      </c>
+      <c r="G40" t="s">
+        <v>185</v>
+      </c>
+      <c r="H40" t="s">
+        <v>25</v>
+      </c>
+      <c r="I40" t="s">
+        <v>25</v>
+      </c>
+      <c r="J40" t="s">
+        <v>25</v>
+      </c>
+      <c r="K40" t="s">
+        <v>25</v>
+      </c>
+      <c r="L40">
+        <v>6799999</v>
+      </c>
+      <c r="M40">
+        <v>4799999</v>
+      </c>
+      <c r="N40" t="s">
+        <v>30</v>
+      </c>
+      <c r="O40" t="s">
+        <v>25</v>
+      </c>
+      <c r="P40">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>76</v>
+      </c>
+      <c r="R40" t="s">
+        <v>68</v>
+      </c>
+      <c r="S40" t="s">
+        <v>33</v>
+      </c>
+      <c r="T40" t="s">
+        <v>99</v>
+      </c>
+      <c r="U40" t="s">
+        <v>100</v>
+      </c>
+      <c r="V40" t="s">
+        <v>101</v>
+      </c>
+      <c r="W40" t="s">
+        <v>25</v>
+      </c>
+      <c r="X40" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y40" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>25</v>
+      </c>
+      <c r="B41" t="s">
+        <v>186</v>
+      </c>
+      <c r="C41" t="s">
+        <v>27</v>
+      </c>
+      <c r="D41" t="s">
+        <v>103</v>
+      </c>
+      <c r="E41" t="s">
+        <v>25</v>
+      </c>
+      <c r="F41">
+        <v>2026</v>
+      </c>
+      <c r="G41" t="s">
+        <v>187</v>
+      </c>
+      <c r="H41" t="s">
+        <v>25</v>
+      </c>
+      <c r="I41" t="s">
+        <v>25</v>
+      </c>
+      <c r="J41" t="s">
+        <v>25</v>
+      </c>
+      <c r="K41" t="s">
+        <v>25</v>
+      </c>
+      <c r="L41">
+        <v>7299998</v>
+      </c>
+      <c r="M41">
+        <v>5299999</v>
+      </c>
+      <c r="N41" t="s">
+        <v>30</v>
+      </c>
+      <c r="O41" t="s">
+        <v>25</v>
+      </c>
+      <c r="P41">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>76</v>
+      </c>
+      <c r="R41" t="s">
+        <v>68</v>
+      </c>
+      <c r="S41" t="s">
+        <v>33</v>
+      </c>
+      <c r="T41" t="s">
+        <v>99</v>
+      </c>
+      <c r="U41" t="s">
+        <v>105</v>
+      </c>
+      <c r="V41" t="s">
+        <v>106</v>
+      </c>
+      <c r="W41" t="s">
+        <v>25</v>
+      </c>
+      <c r="X41" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y41" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>25</v>
+      </c>
+      <c r="B42" t="s">
+        <v>188</v>
+      </c>
+      <c r="C42" t="s">
+        <v>27</v>
+      </c>
+      <c r="D42" t="s">
+        <v>103</v>
+      </c>
+      <c r="E42" t="s">
+        <v>25</v>
+      </c>
+      <c r="F42">
+        <v>2026</v>
+      </c>
+      <c r="G42" t="s">
+        <v>189</v>
+      </c>
+      <c r="H42" t="s">
+        <v>25</v>
+      </c>
+      <c r="I42" t="s">
+        <v>25</v>
+      </c>
+      <c r="J42" t="s">
+        <v>25</v>
+      </c>
+      <c r="K42" t="s">
+        <v>25</v>
+      </c>
+      <c r="L42">
+        <v>7299998</v>
+      </c>
+      <c r="M42">
+        <v>5299999</v>
+      </c>
+      <c r="N42" t="s">
+        <v>30</v>
+      </c>
+      <c r="O42" t="s">
+        <v>25</v>
+      </c>
+      <c r="P42">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>76</v>
+      </c>
+      <c r="R42" t="s">
+        <v>68</v>
+      </c>
+      <c r="S42" t="s">
+        <v>33</v>
+      </c>
+      <c r="T42" t="s">
+        <v>99</v>
+      </c>
+      <c r="U42" t="s">
+        <v>105</v>
+      </c>
+      <c r="V42" t="s">
+        <v>106</v>
+      </c>
+      <c r="W42" t="s">
+        <v>25</v>
+      </c>
+      <c r="X42" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y42" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="43" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>25</v>
+      </c>
+      <c r="B43" t="s">
+        <v>190</v>
+      </c>
+      <c r="C43" t="s">
+        <v>27</v>
+      </c>
+      <c r="D43" t="s">
+        <v>108</v>
+      </c>
+      <c r="E43" t="s">
+        <v>25</v>
+      </c>
+      <c r="F43">
+        <v>2026</v>
+      </c>
+      <c r="G43" t="s">
+        <v>191</v>
+      </c>
+      <c r="H43" t="s">
+        <v>25</v>
+      </c>
+      <c r="I43" t="s">
+        <v>25</v>
+      </c>
+      <c r="J43" t="s">
+        <v>25</v>
+      </c>
+      <c r="K43" t="s">
+        <v>25</v>
+      </c>
+      <c r="L43">
+        <v>7399999</v>
+      </c>
+      <c r="M43">
+        <v>5399999</v>
+      </c>
+      <c r="N43" t="s">
+        <v>30</v>
+      </c>
+      <c r="O43" t="s">
+        <v>25</v>
+      </c>
+      <c r="P43">
+        <v>0</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>76</v>
+      </c>
+      <c r="R43" t="s">
+        <v>110</v>
+      </c>
+      <c r="S43" t="s">
+        <v>33</v>
+      </c>
+      <c r="T43" t="s">
+        <v>111</v>
+      </c>
+      <c r="U43" t="s">
+        <v>112</v>
+      </c>
+      <c r="V43" t="s">
+        <v>113</v>
+      </c>
+      <c r="W43" t="s">
+        <v>25</v>
+      </c>
+      <c r="X43" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y43" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>25</v>
+      </c>
+      <c r="B44" t="s">
+        <v>192</v>
+      </c>
+      <c r="C44" t="s">
+        <v>27</v>
+      </c>
+      <c r="D44" t="s">
+        <v>108</v>
+      </c>
+      <c r="E44" t="s">
+        <v>25</v>
+      </c>
+      <c r="F44">
+        <v>2026</v>
+      </c>
+      <c r="G44" t="s">
+        <v>193</v>
+      </c>
+      <c r="H44" t="s">
+        <v>25</v>
+      </c>
+      <c r="I44" t="s">
+        <v>25</v>
+      </c>
+      <c r="J44" t="s">
+        <v>25</v>
+      </c>
+      <c r="K44" t="s">
+        <v>25</v>
+      </c>
+      <c r="L44">
+        <v>7399999</v>
+      </c>
+      <c r="M44">
+        <v>5399999</v>
+      </c>
+      <c r="N44" t="s">
+        <v>30</v>
+      </c>
+      <c r="O44" t="s">
+        <v>25</v>
+      </c>
+      <c r="P44">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>76</v>
+      </c>
+      <c r="R44" t="s">
+        <v>110</v>
+      </c>
+      <c r="S44" t="s">
+        <v>33</v>
+      </c>
+      <c r="T44" t="s">
+        <v>111</v>
+      </c>
+      <c r="U44" t="s">
+        <v>112</v>
+      </c>
+      <c r="V44" t="s">
+        <v>113</v>
+      </c>
+      <c r="W44" t="s">
+        <v>25</v>
+      </c>
+      <c r="X44" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y44" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>25</v>
+      </c>
+      <c r="B45" t="s">
+        <v>194</v>
+      </c>
+      <c r="C45" t="s">
+        <v>27</v>
+      </c>
+      <c r="D45" t="s">
+        <v>116</v>
+      </c>
+      <c r="E45" t="s">
+        <v>25</v>
+      </c>
+      <c r="F45">
+        <v>2026</v>
+      </c>
+      <c r="G45" t="s">
+        <v>195</v>
+      </c>
+      <c r="H45" t="s">
+        <v>25</v>
+      </c>
+      <c r="I45" t="s">
+        <v>25</v>
+      </c>
+      <c r="J45" t="s">
+        <v>25</v>
+      </c>
+      <c r="K45" t="s">
+        <v>25</v>
+      </c>
+      <c r="L45">
+        <v>10899999</v>
+      </c>
+      <c r="M45">
+        <v>8899999</v>
+      </c>
+      <c r="N45" t="s">
+        <v>30</v>
+      </c>
+      <c r="O45" t="s">
+        <v>25</v>
+      </c>
+      <c r="P45">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>76</v>
+      </c>
+      <c r="R45" t="s">
+        <v>110</v>
+      </c>
+      <c r="S45" t="s">
+        <v>33</v>
+      </c>
+      <c r="T45" t="s">
+        <v>118</v>
+      </c>
+      <c r="U45" t="s">
+        <v>119</v>
+      </c>
+      <c r="V45" t="s">
+        <v>120</v>
+      </c>
+      <c r="W45" t="s">
+        <v>25</v>
+      </c>
+      <c r="X45" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y45" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="46" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>25</v>
+      </c>
+      <c r="B46" t="s">
+        <v>196</v>
+      </c>
+      <c r="C46" t="s">
+        <v>27</v>
+      </c>
+      <c r="D46" t="s">
+        <v>116</v>
+      </c>
+      <c r="E46" t="s">
+        <v>25</v>
+      </c>
+      <c r="F46">
+        <v>2026</v>
+      </c>
+      <c r="G46" t="s">
+        <v>197</v>
+      </c>
+      <c r="H46" t="s">
+        <v>25</v>
+      </c>
+      <c r="I46" t="s">
+        <v>25</v>
+      </c>
+      <c r="J46" t="s">
+        <v>25</v>
+      </c>
+      <c r="K46" t="s">
+        <v>25</v>
+      </c>
+      <c r="L46">
+        <v>10899999</v>
+      </c>
+      <c r="M46">
+        <v>8899999</v>
+      </c>
+      <c r="N46" t="s">
+        <v>30</v>
+      </c>
+      <c r="O46" t="s">
+        <v>25</v>
+      </c>
+      <c r="P46">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>76</v>
+      </c>
+      <c r="R46" t="s">
+        <v>110</v>
+      </c>
+      <c r="S46" t="s">
+        <v>33</v>
+      </c>
+      <c r="T46" t="s">
+        <v>118</v>
+      </c>
+      <c r="U46" t="s">
+        <v>119</v>
+      </c>
+      <c r="V46" t="s">
+        <v>120</v>
+      </c>
+      <c r="W46" t="s">
+        <v>25</v>
+      </c>
+      <c r="X46" t="s">
+        <v>114</v>
+      </c>
+      <c r="Y46" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="47" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>25</v>
+      </c>
+      <c r="B47" t="s">
+        <v>198</v>
+      </c>
+      <c r="C47" t="s">
+        <v>27</v>
+      </c>
+      <c r="D47" t="s">
+        <v>122</v>
+      </c>
+      <c r="E47" t="s">
+        <v>25</v>
+      </c>
+      <c r="F47">
+        <v>2026</v>
+      </c>
+      <c r="G47" t="s">
+        <v>199</v>
+      </c>
+      <c r="H47" t="s">
+        <v>25</v>
+      </c>
+      <c r="I47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J47" t="s">
+        <v>25</v>
+      </c>
+      <c r="K47" t="s">
+        <v>25</v>
+      </c>
+      <c r="L47">
+        <v>3699999</v>
+      </c>
+      <c r="M47">
+        <v>1699999</v>
+      </c>
+      <c r="N47" t="s">
+        <v>30</v>
+      </c>
+      <c r="O47" t="s">
+        <v>25</v>
+      </c>
+      <c r="P47">
+        <v>0</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>76</v>
+      </c>
+      <c r="R47" t="s">
+        <v>124</v>
+      </c>
+      <c r="S47" t="s">
+        <v>33</v>
+      </c>
+      <c r="T47" t="s">
+        <v>125</v>
+      </c>
+      <c r="U47" t="s">
+        <v>126</v>
+      </c>
+      <c r="V47" t="s">
+        <v>127</v>
+      </c>
+      <c r="W47" t="s">
+        <v>25</v>
+      </c>
+      <c r="X47" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y47" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="48" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>25</v>
+      </c>
+      <c r="B48" t="s">
+        <v>200</v>
+      </c>
+      <c r="C48" t="s">
+        <v>27</v>
+      </c>
+      <c r="D48" t="s">
+        <v>122</v>
+      </c>
+      <c r="E48" t="s">
+        <v>25</v>
+      </c>
+      <c r="F48">
+        <v>2026</v>
+      </c>
+      <c r="G48" t="s">
+        <v>201</v>
+      </c>
+      <c r="H48" t="s">
+        <v>25</v>
+      </c>
+      <c r="I48" t="s">
+        <v>25</v>
+      </c>
+      <c r="J48" t="s">
+        <v>25</v>
+      </c>
+      <c r="K48" t="s">
+        <v>25</v>
+      </c>
+      <c r="L48">
+        <v>3699999</v>
+      </c>
+      <c r="M48">
+        <v>1699999</v>
+      </c>
+      <c r="N48" t="s">
+        <v>30</v>
+      </c>
+      <c r="O48" t="s">
+        <v>25</v>
+      </c>
+      <c r="P48">
+        <v>0</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>76</v>
+      </c>
+      <c r="R48" t="s">
+        <v>124</v>
+      </c>
+      <c r="S48" t="s">
+        <v>33</v>
+      </c>
+      <c r="T48" t="s">
+        <v>125</v>
+      </c>
+      <c r="U48" t="s">
+        <v>126</v>
+      </c>
+      <c r="V48" t="s">
+        <v>127</v>
+      </c>
+      <c r="W48" t="s">
+        <v>25</v>
+      </c>
+      <c r="X48" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y48" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="49" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>25</v>
+      </c>
+      <c r="B49" t="s">
+        <v>202</v>
+      </c>
+      <c r="C49" t="s">
+        <v>27</v>
+      </c>
+      <c r="D49" t="s">
+        <v>130</v>
+      </c>
+      <c r="E49" t="s">
+        <v>25</v>
+      </c>
+      <c r="F49">
+        <v>2026</v>
+      </c>
+      <c r="G49" t="s">
+        <v>203</v>
+      </c>
+      <c r="H49" t="s">
+        <v>25</v>
+      </c>
+      <c r="I49" t="s">
+        <v>25</v>
+      </c>
+      <c r="J49" t="s">
+        <v>25</v>
+      </c>
+      <c r="K49" t="s">
+        <v>25</v>
+      </c>
+      <c r="L49">
+        <v>3899998</v>
+      </c>
+      <c r="M49">
+        <v>1899999</v>
+      </c>
+      <c r="N49" t="s">
+        <v>30</v>
+      </c>
+      <c r="O49" t="s">
+        <v>25</v>
+      </c>
+      <c r="P49">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>76</v>
+      </c>
+      <c r="R49" t="s">
+        <v>124</v>
+      </c>
+      <c r="S49" t="s">
+        <v>33</v>
+      </c>
+      <c r="T49" t="s">
+        <v>125</v>
+      </c>
+      <c r="U49" t="s">
+        <v>132</v>
+      </c>
+      <c r="V49" t="s">
+        <v>133</v>
+      </c>
+      <c r="W49" t="s">
+        <v>25</v>
+      </c>
+      <c r="X49" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y49" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="50" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>25</v>
+      </c>
+      <c r="B50" t="s">
+        <v>204</v>
+      </c>
+      <c r="C50" t="s">
+        <v>27</v>
+      </c>
+      <c r="D50" t="s">
+        <v>130</v>
+      </c>
+      <c r="E50" t="s">
+        <v>25</v>
+      </c>
+      <c r="F50">
+        <v>2026</v>
+      </c>
+      <c r="G50" t="s">
+        <v>205</v>
+      </c>
+      <c r="H50" t="s">
+        <v>25</v>
+      </c>
+      <c r="I50" t="s">
+        <v>25</v>
+      </c>
+      <c r="J50" t="s">
+        <v>25</v>
+      </c>
+      <c r="K50" t="s">
+        <v>25</v>
+      </c>
+      <c r="L50">
+        <v>3899998</v>
+      </c>
+      <c r="M50">
+        <v>1899999</v>
+      </c>
+      <c r="N50" t="s">
+        <v>30</v>
+      </c>
+      <c r="O50" t="s">
+        <v>25</v>
+      </c>
+      <c r="P50">
+        <v>0</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>76</v>
+      </c>
+      <c r="R50" t="s">
+        <v>124</v>
+      </c>
+      <c r="S50" t="s">
+        <v>33</v>
+      </c>
+      <c r="T50" t="s">
+        <v>125</v>
+      </c>
+      <c r="U50" t="s">
+        <v>132</v>
+      </c>
+      <c r="V50" t="s">
+        <v>133</v>
+      </c>
+      <c r="W50" t="s">
+        <v>25</v>
+      </c>
+      <c r="X50" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y50" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>25</v>
+      </c>
+      <c r="B51" t="s">
+        <v>206</v>
+      </c>
+      <c r="C51" t="s">
+        <v>27</v>
+      </c>
+      <c r="D51" t="s">
+        <v>135</v>
+      </c>
+      <c r="E51" t="s">
+        <v>25</v>
+      </c>
+      <c r="F51">
+        <v>2026</v>
+      </c>
+      <c r="G51" t="s">
+        <v>207</v>
+      </c>
+      <c r="H51" t="s">
+        <v>25</v>
+      </c>
+      <c r="I51" t="s">
+        <v>25</v>
+      </c>
+      <c r="J51" t="s">
+        <v>25</v>
+      </c>
+      <c r="K51" t="s">
+        <v>25</v>
+      </c>
+      <c r="L51">
+        <v>4799999</v>
+      </c>
+      <c r="M51">
+        <v>2799999</v>
+      </c>
+      <c r="N51" t="s">
+        <v>30</v>
+      </c>
+      <c r="O51" t="s">
+        <v>25</v>
+      </c>
+      <c r="P51">
+        <v>0</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>76</v>
+      </c>
+      <c r="R51" t="s">
+        <v>124</v>
+      </c>
+      <c r="S51" t="s">
+        <v>33</v>
+      </c>
+      <c r="T51" t="s">
+        <v>125</v>
+      </c>
+      <c r="U51" t="s">
+        <v>137</v>
+      </c>
+      <c r="V51" t="s">
+        <v>138</v>
+      </c>
+      <c r="W51" t="s">
+        <v>25</v>
+      </c>
+      <c r="X51" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y51" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="52" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>25</v>
+      </c>
+      <c r="B52" t="s">
+        <v>208</v>
+      </c>
+      <c r="C52" t="s">
+        <v>27</v>
+      </c>
+      <c r="D52" t="s">
+        <v>135</v>
+      </c>
+      <c r="E52" t="s">
+        <v>25</v>
+      </c>
+      <c r="F52">
+        <v>2026</v>
+      </c>
+      <c r="G52" t="s">
+        <v>209</v>
+      </c>
+      <c r="H52" t="s">
+        <v>25</v>
+      </c>
+      <c r="I52" t="s">
+        <v>25</v>
+      </c>
+      <c r="J52" t="s">
+        <v>25</v>
+      </c>
+      <c r="K52" t="s">
+        <v>25</v>
+      </c>
+      <c r="L52">
+        <v>4799999</v>
+      </c>
+      <c r="M52">
+        <v>2799999</v>
+      </c>
+      <c r="N52" t="s">
+        <v>30</v>
+      </c>
+      <c r="O52" t="s">
+        <v>25</v>
+      </c>
+      <c r="P52">
+        <v>0</v>
+      </c>
+      <c r="Q52" t="s">
+        <v>76</v>
+      </c>
+      <c r="R52" t="s">
+        <v>124</v>
+      </c>
+      <c r="S52" t="s">
+        <v>33</v>
+      </c>
+      <c r="T52" t="s">
+        <v>125</v>
+      </c>
+      <c r="U52" t="s">
+        <v>137</v>
+      </c>
+      <c r="V52" t="s">
+        <v>138</v>
+      </c>
+      <c r="W52" t="s">
+        <v>25</v>
+      </c>
+      <c r="X52" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y52" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>